<commit_message>
Add Contact Energy logo and footer to all xlsx templates
add_branding.py post-processes every xlsx in the project (except
New_Relay_Onboarding_Form): inserts the Contact_2020_Master_RGB_Gradient
logo (87×40 px, 2.18:1 aspect) anchored top-right of the title row on
every worksheet, and a print footer on every sheet:
  Left:   Bold "Contact Energy" in brand blue (#1F4E79), 8 pt
  Centre: Document name (filename without extension), 8 pt
  Right:  "Page X of Y", 8 pt

Covers 12 files × 1-9 sheets = 111 worksheets total. Idempotent —
clears previous logos before re-adding so the script is safe to rerun.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ABB_Biennial_Visual_Check.xlsx
+++ b/ABB_Biennial_Visual_Check.xlsx
@@ -105,7 +105,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -119,11 +119,74 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -171,6 +234,15 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -245,6 +317,66 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="828675" cy="381000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="828675" cy="381000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -559,6 +691,10 @@
           <t>1.  IED AND SITE INFORMATION</t>
         </is>
       </c>
+      <c r="B3" s="17" t="n"/>
+      <c r="C3" s="17" t="n"/>
+      <c r="D3" s="17" t="n"/>
+      <c r="E3" s="18" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -571,6 +707,9 @@
           <t>REG670  /  RET670  (circle one)</t>
         </is>
       </c>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="18" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -579,6 +718,9 @@
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -587,6 +729,9 @@
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -595,6 +740,9 @@
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="18" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -603,6 +751,9 @@
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="18" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -611,6 +762,9 @@
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="18" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -619,6 +773,9 @@
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="18" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -627,6 +784,9 @@
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="18" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -639,6 +799,9 @@
           <t>(2 years from date above)</t>
         </is>
       </c>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="18" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -646,6 +809,10 @@
           <t>2.  CONNECTION METHOD</t>
         </is>
       </c>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="18" t="n"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -655,6 +822,10 @@
 OPTION C — Ethernet + web browser: Navigate to IED IP address in browser (if web server enabled).</t>
         </is>
       </c>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="18" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -667,6 +838,9 @@
           <t>LHMI only  /  Ethernet + PCM600  /  Ethernet + browser  (delete as applicable)</t>
         </is>
       </c>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="18" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -674,6 +848,10 @@
           <t>3.  SELF-TEST AND IED STATUS  (INTERRSIG self-supervision)</t>
         </is>
       </c>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="18" t="n"/>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -681,6 +859,10 @@
           <t>LHMI path: Main menu → Diagnostics → IED status → Signals → INTERRSIG.  All signals should show NORMAL (0). A FAIL signal asserts the INTERNAL FAIL contact on the PSM. Hardware modules: Main menu → Diagnostics → Hardware → Module status.</t>
         </is>
       </c>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="18" t="n"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -924,6 +1106,10 @@
           <t>4.  ANALOGUE MEASUREMENTS  (Primary Values)</t>
         </is>
       </c>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="17" t="n"/>
+      <c r="D33" s="17" t="n"/>
+      <c r="E33" s="18" t="n"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -931,6 +1117,10 @@
           <t>LHMI: Main menu → Measurements → [function block, e.g. T2WPDIF, GENPDIF, OC4PTOC] → monitored data.  All values displayed in primary units. Record current load values below.  PCM600: Signal Monitor shows live primary values.</t>
         </is>
       </c>
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="17" t="n"/>
+      <c r="D34" s="17" t="n"/>
+      <c r="E34" s="18" t="n"/>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
@@ -1148,6 +1338,10 @@
           <t>5.  CLOCK AND TIME SYNCHRONISATION</t>
         </is>
       </c>
+      <c r="B47" s="17" t="n"/>
+      <c r="C47" s="17" t="n"/>
+      <c r="D47" s="17" t="n"/>
+      <c r="E47" s="18" t="n"/>
     </row>
     <row r="48" ht="28" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
@@ -1259,6 +1453,10 @@
           <t>6.  RECENT EVENTS  (record most recent disturbance records / events)</t>
         </is>
       </c>
+      <c r="B54" s="17" t="n"/>
+      <c r="C54" s="17" t="n"/>
+      <c r="D54" s="17" t="n"/>
+      <c r="E54" s="18" t="n"/>
     </row>
     <row r="55" ht="32" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
@@ -1266,6 +1464,10 @@
           <t>LHMI: Main menu → Events → Disturbance records list (most recent first).  PCM600: Event viewer shows all logged events with timestamps.  Record the most recent events; flag any unexplained trips or alarms.</t>
         </is>
       </c>
+      <c r="B55" s="17" t="n"/>
+      <c r="C55" s="17" t="n"/>
+      <c r="D55" s="17" t="n"/>
+      <c r="E55" s="18" t="n"/>
     </row>
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
@@ -1289,6 +1491,7 @@
           <t>Event Description / Type</t>
         </is>
       </c>
+      <c r="E56" s="18" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
@@ -1297,6 +1500,7 @@
       <c r="B57" s="4" t="n"/>
       <c r="C57" s="4" t="n"/>
       <c r="D57" s="4" t="n"/>
+      <c r="E57" s="18" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="12" t="n">
@@ -1305,6 +1509,7 @@
       <c r="B58" s="13" t="n"/>
       <c r="C58" s="13" t="n"/>
       <c r="D58" s="13" t="n"/>
+      <c r="E58" s="18" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
@@ -1313,6 +1518,7 @@
       <c r="B59" s="4" t="n"/>
       <c r="C59" s="4" t="n"/>
       <c r="D59" s="4" t="n"/>
+      <c r="E59" s="18" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="n">
@@ -1321,6 +1527,7 @@
       <c r="B60" s="13" t="n"/>
       <c r="C60" s="13" t="n"/>
       <c r="D60" s="13" t="n"/>
+      <c r="E60" s="18" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
@@ -1329,6 +1536,7 @@
       <c r="B61" s="4" t="n"/>
       <c r="C61" s="4" t="n"/>
       <c r="D61" s="4" t="n"/>
+      <c r="E61" s="18" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="n">
@@ -1337,6 +1545,7 @@
       <c r="B62" s="13" t="n"/>
       <c r="C62" s="13" t="n"/>
       <c r="D62" s="13" t="n"/>
+      <c r="E62" s="18" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
@@ -1345,6 +1554,7 @@
       <c r="B63" s="4" t="n"/>
       <c r="C63" s="4" t="n"/>
       <c r="D63" s="4" t="n"/>
+      <c r="E63" s="18" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="n">
@@ -1353,6 +1563,7 @@
       <c r="B64" s="13" t="n"/>
       <c r="C64" s="13" t="n"/>
       <c r="D64" s="13" t="n"/>
+      <c r="E64" s="18" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
@@ -1361,6 +1572,7 @@
       <c r="B65" s="4" t="n"/>
       <c r="C65" s="4" t="n"/>
       <c r="D65" s="4" t="n"/>
+      <c r="E65" s="18" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="12" t="n">
@@ -1369,6 +1581,7 @@
       <c r="B66" s="13" t="n"/>
       <c r="C66" s="13" t="n"/>
       <c r="D66" s="13" t="n"/>
+      <c r="E66" s="18" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n">
@@ -1377,6 +1590,7 @@
       <c r="B67" s="4" t="n"/>
       <c r="C67" s="4" t="n"/>
       <c r="D67" s="4" t="n"/>
+      <c r="E67" s="18" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="12" t="n">
@@ -1385,6 +1599,7 @@
       <c r="B68" s="13" t="n"/>
       <c r="C68" s="13" t="n"/>
       <c r="D68" s="13" t="n"/>
+      <c r="E68" s="18" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -1393,6 +1608,9 @@
         </is>
       </c>
       <c r="B69" s="4" t="n"/>
+      <c r="C69" s="17" t="n"/>
+      <c r="D69" s="17" t="n"/>
+      <c r="E69" s="18" t="n"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
@@ -1400,6 +1618,10 @@
           <t>7.  DCS / ABB 800XA COMMUNICATION CHECK</t>
         </is>
       </c>
+      <c r="B71" s="17" t="n"/>
+      <c r="C71" s="17" t="n"/>
+      <c r="D71" s="17" t="n"/>
+      <c r="E71" s="18" t="n"/>
     </row>
     <row r="72" ht="36" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
@@ -1407,6 +1629,10 @@
           <t>Open the IED faceplate in the ABB 800XA control system. Verify live values (currents, IED status indicators) are updating. The 800XA communicates via IEC 61850 GOOSE / MMS. No yellow or red communication alarm objects should be present.</t>
         </is>
       </c>
+      <c r="B72" s="17" t="n"/>
+      <c r="C72" s="17" t="n"/>
+      <c r="D72" s="17" t="n"/>
+      <c r="E72" s="18" t="n"/>
     </row>
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
@@ -1430,6 +1656,7 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="E73" s="18" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -1444,6 +1671,7 @@
       </c>
       <c r="C74" s="10" t="n"/>
       <c r="D74" s="4" t="n"/>
+      <c r="E74" s="18" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -1458,6 +1686,7 @@
       </c>
       <c r="C75" s="10" t="n"/>
       <c r="D75" s="4" t="n"/>
+      <c r="E75" s="18" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -1472,6 +1701,7 @@
       </c>
       <c r="C76" s="10" t="n"/>
       <c r="D76" s="4" t="n"/>
+      <c r="E76" s="18" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -1486,6 +1716,7 @@
       </c>
       <c r="C77" s="10" t="n"/>
       <c r="D77" s="4" t="n"/>
+      <c r="E77" s="18" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -1500,6 +1731,7 @@
       </c>
       <c r="C78" s="10" t="n"/>
       <c r="D78" s="4" t="n"/>
+      <c r="E78" s="18" t="n"/>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
@@ -1507,6 +1739,10 @@
           <t>8.  OPTIONAL — CLEAR EVENT BUFFERS  (only if required by your procedure)</t>
         </is>
       </c>
+      <c r="B80" s="17" t="n"/>
+      <c r="C80" s="17" t="n"/>
+      <c r="D80" s="17" t="n"/>
+      <c r="E80" s="18" t="n"/>
     </row>
     <row r="81" ht="36" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
@@ -1514,6 +1750,10 @@
           <t>Only clear events if required by site procedure. Ensure all events have been downloaded/recorded BEFORE clearing. LHMI: Main menu → Events → [select event] → Clear  (or Clear all).  Internal events (INTERRSIG log) clear automatically after 40 events (FIFO).</t>
         </is>
       </c>
+      <c r="B81" s="17" t="n"/>
+      <c r="C81" s="17" t="n"/>
+      <c r="D81" s="17" t="n"/>
+      <c r="E81" s="18" t="n"/>
     </row>
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
@@ -1537,6 +1777,7 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="E82" s="18" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -1551,6 +1792,7 @@
       </c>
       <c r="C83" s="10" t="n"/>
       <c r="D83" s="4" t="n"/>
+      <c r="E83" s="18" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -1565,6 +1807,7 @@
       </c>
       <c r="C84" s="10" t="n"/>
       <c r="D84" s="4" t="n"/>
+      <c r="E84" s="18" t="n"/>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
@@ -1572,30 +1815,32 @@
           <t>9.  OBSERVATIONS AND CORRECTIVE ACTIONS</t>
         </is>
       </c>
+      <c r="B86" s="17" t="n"/>
+      <c r="C86" s="17" t="n"/>
+      <c r="D86" s="17" t="n"/>
+      <c r="E86" s="18" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="15" t="n"/>
+      <c r="B87" s="19" t="n"/>
+      <c r="C87" s="19" t="n"/>
+      <c r="D87" s="19" t="n"/>
+      <c r="E87" s="20" t="n"/>
     </row>
     <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="16" t="n"/>
-      <c r="B88" s="16" t="n"/>
-      <c r="C88" s="16" t="n"/>
-      <c r="D88" s="16" t="n"/>
-      <c r="E88" s="16" t="n"/>
+      <c r="A88" s="21" t="n"/>
+      <c r="E88" s="22" t="n"/>
     </row>
     <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="16" t="n"/>
-      <c r="B89" s="16" t="n"/>
-      <c r="C89" s="16" t="n"/>
-      <c r="D89" s="16" t="n"/>
-      <c r="E89" s="16" t="n"/>
+      <c r="A89" s="21" t="n"/>
+      <c r="E89" s="22" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="16" t="n"/>
-      <c r="B90" s="16" t="n"/>
-      <c r="C90" s="16" t="n"/>
-      <c r="D90" s="16" t="n"/>
-      <c r="E90" s="16" t="n"/>
+      <c r="A90" s="23" t="n"/>
+      <c r="B90" s="24" t="n"/>
+      <c r="C90" s="24" t="n"/>
+      <c r="D90" s="24" t="n"/>
+      <c r="E90" s="25" t="n"/>
     </row>
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
@@ -1603,6 +1848,10 @@
           <t>10.  SIGN-OFF</t>
         </is>
       </c>
+      <c r="B92" s="17" t="n"/>
+      <c r="C92" s="17" t="n"/>
+      <c r="D92" s="17" t="n"/>
+      <c r="E92" s="18" t="n"/>
     </row>
     <row r="93" ht="28" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
@@ -1625,6 +1874,7 @@
           <t>Date</t>
         </is>
       </c>
+      <c r="E93" s="18" t="n"/>
     </row>
     <row r="94" ht="24" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
@@ -1635,6 +1885,7 @@
       <c r="B94" s="4" t="n"/>
       <c r="C94" s="4" t="n"/>
       <c r="D94" s="4" t="n"/>
+      <c r="E94" s="18" t="n"/>
     </row>
     <row r="95" ht="24" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
@@ -1645,12 +1896,13 @@
       <c r="B95" s="4" t="n"/>
       <c r="C95" s="4" t="n"/>
       <c r="D95" s="4" t="n"/>
+      <c r="E95" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="54">
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="D60:E60"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="D60:E60"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="D63:E63"/>
     <mergeCell ref="B6:E6"/>
@@ -1705,6 +1957,15 @@
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;8 &amp;K1F4E79&amp;BContact Energy&amp;C&amp;8 ABB Biennial Visual Check&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter>&amp;L&amp;8 &amp;K1F4E79&amp;BContact Energy&amp;C&amp;8 ABB Biennial Visual Check&amp;R&amp;8 Page &amp;P of &amp;N</evenFooter>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1737,6 +1998,10 @@
           <t>1.  IED AND SITE INFORMATION</t>
         </is>
       </c>
+      <c r="B3" s="17" t="n"/>
+      <c r="C3" s="17" t="n"/>
+      <c r="D3" s="17" t="n"/>
+      <c r="E3" s="18" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1749,6 +2014,9 @@
           <t>REF615  /  RET615  /  REM615  /  REU615  (circle one)</t>
         </is>
       </c>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="18" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1757,6 +2025,9 @@
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1765,6 +2036,9 @@
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1773,6 +2047,9 @@
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="18" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1781,6 +2058,9 @@
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="18" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1789,6 +2069,9 @@
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="18" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1797,6 +2080,9 @@
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="18" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1805,6 +2091,9 @@
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="18" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1817,6 +2106,9 @@
           <t>(2 years from date above)</t>
         </is>
       </c>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="18" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1824,6 +2116,10 @@
           <t>2.  CONNECTION METHOD</t>
         </is>
       </c>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="18" t="n"/>
     </row>
     <row r="15" ht="64" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1833,6 +2129,10 @@
 OPTION C — Ethernet + web browser: Newer 615 C/D models support a built-in web server — navigate to IED IP address in a browser.</t>
         </is>
       </c>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="18" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1845,6 +2145,9 @@
           <t>LHMI only  /  Ethernet + PCM600  /  Ethernet + browser  (delete as applicable)</t>
         </is>
       </c>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="18" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1852,6 +2155,10 @@
           <t>3.  SELF-TEST AND IED STATUS</t>
         </is>
       </c>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="18" t="n"/>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1859,6 +2166,10 @@
           <t>Key LED indicators on front panel:  READY (green, solid) = IED healthy and in service.  START (yellow) = protection element picked up (may be normal under load).  TRIP (red) = protection has tripped.  Self-supervision: LHMI: Main menu → Monitoring → Self-supervision → IED status.</t>
         </is>
       </c>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="18" t="n"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -2026,6 +2337,10 @@
           <t>4.  ANALOGUE MEASUREMENTS  (Primary Values)</t>
         </is>
       </c>
+      <c r="B29" s="17" t="n"/>
+      <c r="C29" s="17" t="n"/>
+      <c r="D29" s="17" t="n"/>
+      <c r="E29" s="18" t="n"/>
     </row>
     <row r="30" ht="40" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -2033,6 +2348,10 @@
           <t>LHMI: Main menu → Monitoring → Measurements → Current (or Voltage).  All values shown in primary units. PCM600 Signal Monitor also displays live primary values.  Record current values. Flag anything obviously abnormal (e.g. one phase zero while others are loaded).</t>
         </is>
       </c>
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="17" t="n"/>
+      <c r="D30" s="17" t="n"/>
+      <c r="E30" s="18" t="n"/>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
@@ -2221,6 +2540,10 @@
           <t>5.  CLOCK AND TIME SYNCHRONISATION</t>
         </is>
       </c>
+      <c r="B41" s="17" t="n"/>
+      <c r="C41" s="17" t="n"/>
+      <c r="D41" s="17" t="n"/>
+      <c r="E41" s="18" t="n"/>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
@@ -2313,6 +2636,10 @@
           <t>6.  RECENT EVENTS  (record most recent events from the event list)</t>
         </is>
       </c>
+      <c r="B47" s="17" t="n"/>
+      <c r="C47" s="17" t="n"/>
+      <c r="D47" s="17" t="n"/>
+      <c r="E47" s="18" t="n"/>
     </row>
     <row r="48" ht="28" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -2320,6 +2647,10 @@
           <t>LHMI: Main menu → Events → Event list (most recent first).  PCM600: Event viewer.  Record the most recent events. Flag any unexplained TRIP or FAULT events.</t>
         </is>
       </c>
+      <c r="B48" s="17" t="n"/>
+      <c r="C48" s="17" t="n"/>
+      <c r="D48" s="17" t="n"/>
+      <c r="E48" s="18" t="n"/>
     </row>
     <row r="49" ht="28" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
@@ -2343,6 +2674,7 @@
           <t>Event Description / Type</t>
         </is>
       </c>
+      <c r="E49" s="18" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n">
@@ -2351,6 +2683,7 @@
       <c r="B50" s="4" t="n"/>
       <c r="C50" s="4" t="n"/>
       <c r="D50" s="4" t="n"/>
+      <c r="E50" s="18" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="12" t="n">
@@ -2359,6 +2692,7 @@
       <c r="B51" s="13" t="n"/>
       <c r="C51" s="13" t="n"/>
       <c r="D51" s="13" t="n"/>
+      <c r="E51" s="18" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
@@ -2367,6 +2701,7 @@
       <c r="B52" s="4" t="n"/>
       <c r="C52" s="4" t="n"/>
       <c r="D52" s="4" t="n"/>
+      <c r="E52" s="18" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="12" t="n">
@@ -2375,6 +2710,7 @@
       <c r="B53" s="13" t="n"/>
       <c r="C53" s="13" t="n"/>
       <c r="D53" s="13" t="n"/>
+      <c r="E53" s="18" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
@@ -2383,6 +2719,7 @@
       <c r="B54" s="4" t="n"/>
       <c r="C54" s="4" t="n"/>
       <c r="D54" s="4" t="n"/>
+      <c r="E54" s="18" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="12" t="n">
@@ -2391,6 +2728,7 @@
       <c r="B55" s="13" t="n"/>
       <c r="C55" s="13" t="n"/>
       <c r="D55" s="13" t="n"/>
+      <c r="E55" s="18" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
@@ -2399,6 +2737,7 @@
       <c r="B56" s="4" t="n"/>
       <c r="C56" s="4" t="n"/>
       <c r="D56" s="4" t="n"/>
+      <c r="E56" s="18" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="12" t="n">
@@ -2407,6 +2746,7 @@
       <c r="B57" s="13" t="n"/>
       <c r="C57" s="13" t="n"/>
       <c r="D57" s="13" t="n"/>
+      <c r="E57" s="18" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
@@ -2415,6 +2755,7 @@
       <c r="B58" s="4" t="n"/>
       <c r="C58" s="4" t="n"/>
       <c r="D58" s="4" t="n"/>
+      <c r="E58" s="18" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="12" t="n">
@@ -2423,6 +2764,7 @@
       <c r="B59" s="13" t="n"/>
       <c r="C59" s="13" t="n"/>
       <c r="D59" s="13" t="n"/>
+      <c r="E59" s="18" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
@@ -2431,6 +2773,7 @@
       <c r="B60" s="4" t="n"/>
       <c r="C60" s="4" t="n"/>
       <c r="D60" s="4" t="n"/>
+      <c r="E60" s="18" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="12" t="n">
@@ -2439,6 +2782,7 @@
       <c r="B61" s="13" t="n"/>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
+      <c r="E61" s="18" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -2447,6 +2791,9 @@
         </is>
       </c>
       <c r="B62" s="4" t="n"/>
+      <c r="C62" s="17" t="n"/>
+      <c r="D62" s="17" t="n"/>
+      <c r="E62" s="18" t="n"/>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -2454,6 +2801,10 @@
           <t>7.  DCS / ABB 800XA COMMUNICATION CHECK</t>
         </is>
       </c>
+      <c r="B64" s="17" t="n"/>
+      <c r="C64" s="17" t="n"/>
+      <c r="D64" s="17" t="n"/>
+      <c r="E64" s="18" t="n"/>
     </row>
     <row r="65" ht="36" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
@@ -2461,6 +2812,10 @@
           <t>Open the IED faceplate in the ABB 800XA control system. Verify live values and IED status are updating. The 615 series typically communicates via IEC 61850, DNP3.0, or Modbus.  No yellow or red communication alarm objects should be present on the 800XA faceplate.</t>
         </is>
       </c>
+      <c r="B65" s="17" t="n"/>
+      <c r="C65" s="17" t="n"/>
+      <c r="D65" s="17" t="n"/>
+      <c r="E65" s="18" t="n"/>
     </row>
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
@@ -2484,6 +2839,7 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="E66" s="18" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -2498,6 +2854,7 @@
       </c>
       <c r="C67" s="10" t="n"/>
       <c r="D67" s="4" t="n"/>
+      <c r="E67" s="18" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -2512,6 +2869,7 @@
       </c>
       <c r="C68" s="10" t="n"/>
       <c r="D68" s="4" t="n"/>
+      <c r="E68" s="18" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -2526,6 +2884,7 @@
       </c>
       <c r="C69" s="10" t="n"/>
       <c r="D69" s="4" t="n"/>
+      <c r="E69" s="18" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -2540,6 +2899,7 @@
       </c>
       <c r="C70" s="10" t="n"/>
       <c r="D70" s="4" t="n"/>
+      <c r="E70" s="18" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -2554,6 +2914,7 @@
       </c>
       <c r="C71" s="10" t="n"/>
       <c r="D71" s="4" t="n"/>
+      <c r="E71" s="18" t="n"/>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
@@ -2561,6 +2922,10 @@
           <t>8.  OPTIONAL — CLEAR EVENTS  (only if required by your procedure)</t>
         </is>
       </c>
+      <c r="B73" s="17" t="n"/>
+      <c r="C73" s="17" t="n"/>
+      <c r="D73" s="17" t="n"/>
+      <c r="E73" s="18" t="n"/>
     </row>
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="14" t="inlineStr">
@@ -2568,6 +2933,10 @@
           <t>Only clear events if required by site procedure. Download/record all events BEFORE clearing. LHMI: Main menu → Events → Event list → Clear all (or select individual events).</t>
         </is>
       </c>
+      <c r="B74" s="17" t="n"/>
+      <c r="C74" s="17" t="n"/>
+      <c r="D74" s="17" t="n"/>
+      <c r="E74" s="18" t="n"/>
     </row>
     <row r="75" ht="28" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
@@ -2591,6 +2960,7 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="E75" s="18" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -2605,6 +2975,7 @@
       </c>
       <c r="C76" s="10" t="n"/>
       <c r="D76" s="4" t="n"/>
+      <c r="E76" s="18" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -2619,6 +2990,7 @@
       </c>
       <c r="C77" s="10" t="n"/>
       <c r="D77" s="4" t="n"/>
+      <c r="E77" s="18" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
@@ -2626,30 +2998,32 @@
           <t>9.  OBSERVATIONS AND CORRECTIVE ACTIONS</t>
         </is>
       </c>
+      <c r="B79" s="17" t="n"/>
+      <c r="C79" s="17" t="n"/>
+      <c r="D79" s="17" t="n"/>
+      <c r="E79" s="18" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="15" t="n"/>
+      <c r="B80" s="19" t="n"/>
+      <c r="C80" s="19" t="n"/>
+      <c r="D80" s="19" t="n"/>
+      <c r="E80" s="20" t="n"/>
     </row>
     <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="16" t="n"/>
-      <c r="B81" s="16" t="n"/>
-      <c r="C81" s="16" t="n"/>
-      <c r="D81" s="16" t="n"/>
-      <c r="E81" s="16" t="n"/>
+      <c r="A81" s="21" t="n"/>
+      <c r="E81" s="22" t="n"/>
     </row>
     <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="16" t="n"/>
-      <c r="B82" s="16" t="n"/>
-      <c r="C82" s="16" t="n"/>
-      <c r="D82" s="16" t="n"/>
-      <c r="E82" s="16" t="n"/>
+      <c r="A82" s="21" t="n"/>
+      <c r="E82" s="22" t="n"/>
     </row>
     <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="16" t="n"/>
-      <c r="B83" s="16" t="n"/>
-      <c r="C83" s="16" t="n"/>
-      <c r="D83" s="16" t="n"/>
-      <c r="E83" s="16" t="n"/>
+      <c r="A83" s="23" t="n"/>
+      <c r="B83" s="24" t="n"/>
+      <c r="C83" s="24" t="n"/>
+      <c r="D83" s="24" t="n"/>
+      <c r="E83" s="25" t="n"/>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
@@ -2657,6 +3031,10 @@
           <t>10.  SIGN-OFF</t>
         </is>
       </c>
+      <c r="B85" s="17" t="n"/>
+      <c r="C85" s="17" t="n"/>
+      <c r="D85" s="17" t="n"/>
+      <c r="E85" s="18" t="n"/>
     </row>
     <row r="86" ht="28" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
@@ -2679,6 +3057,7 @@
           <t>Date</t>
         </is>
       </c>
+      <c r="E86" s="18" t="n"/>
     </row>
     <row r="87" ht="24" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
@@ -2689,6 +3068,7 @@
       <c r="B87" s="4" t="n"/>
       <c r="C87" s="4" t="n"/>
       <c r="D87" s="4" t="n"/>
+      <c r="E87" s="18" t="n"/>
     </row>
     <row r="88" ht="24" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
@@ -2699,13 +3079,14 @@
       <c r="B88" s="4" t="n"/>
       <c r="C88" s="4" t="n"/>
       <c r="D88" s="4" t="n"/>
+      <c r="E88" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="54">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="D69:E69"/>
+    <mergeCell ref="D60:E60"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="D60:E60"/>
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="A73:E73"/>
     <mergeCell ref="A15:E15"/>
@@ -2759,5 +3140,14 @@
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;8 &amp;K1F4E79&amp;BContact Energy&amp;C&amp;8 ABB Biennial Visual Check&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter>&amp;L&amp;8 &amp;K1F4E79&amp;BContact Energy&amp;C&amp;8 ABB Biennial Visual Check&amp;R&amp;8 Page &amp;P of &amp;N</evenFooter>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>